<commit_message>
Move Quarto vignettes to pkgdown articles, remove generated outputs, and standardize PKML filenames
</commit_message>
<xml_diff>
--- a/inst/extdata/Obach1999_IVIVE_input.xlsx
+++ b/inst/extdata/Obach1999_IVIVE_input.xlsx
@@ -301,7 +301,7 @@
     <t xml:space="preserve">observed</t>
   </si>
   <si>
-    <t xml:space="preserve">single IV-PKSim.pkml</t>
+    <t xml:space="preserve">single-iv-pksim.pkml</t>
   </si>
   <si>
     <t xml:space="preserve">S2</t>
@@ -340,7 +340,7 @@
     <t xml:space="preserve">Rodgers &amp; Rowland + fu</t>
   </si>
   <si>
-    <t xml:space="preserve">single IV-R&amp;R.pkml</t>
+    <t xml:space="preserve">single-iv-rodgers-rowland.pkml</t>
   </si>
   <si>
     <t xml:space="preserve">S6</t>

</xml_diff>

<commit_message>
Update README, articles and the Obach sheet to the new names
- README.Rmd, README.md:
  - function list of the 12 exports
  - midazolam example with the new names
  - note on snake_case in the coding standards
- vignettes/articles/*.qmd: new method values and arguments
- dev/make_obach_ivive_sheet.R, inst/extdata/Obach1999_IVIVE_input.xlsx: new method values, logical empirical_correction column
</commit_message>
<xml_diff>
--- a/inst/extdata/Obach1999_IVIVE_input.xlsx
+++ b/inst/extdata/Obach1999_IVIVE_input.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="153">
   <si>
     <t xml:space="preserve">Drug</t>
   </si>
@@ -274,7 +274,7 @@
     <t xml:space="preserve">permeability_high_cmmin</t>
   </si>
   <si>
-    <t xml:space="preserve">empirical_scalar</t>
+    <t xml:space="preserve">empirical_correction</t>
   </si>
   <si>
     <t xml:space="preserve">blood_plasma_ratio</t>
@@ -295,9 +295,6 @@
     <t xml:space="preserve">QSAR</t>
   </si>
   <si>
-    <t xml:space="preserve">No</t>
-  </si>
-  <si>
     <t xml:space="preserve">observed</t>
   </si>
   <si>
@@ -307,16 +304,16 @@
     <t xml:space="preserve">S2</t>
   </si>
   <si>
-    <t xml:space="preserve">fu_mic All_literature, PK-Sim partitioning, QSAR permeability</t>
-  </si>
-  <si>
-    <t xml:space="preserve">All_literature</t>
+    <t xml:space="preserve">fu_mic all_literature, PK-Sim partitioning, QSAR permeability</t>
+  </si>
+  <si>
+    <t xml:space="preserve">all_literature</t>
   </si>
   <si>
     <t xml:space="preserve">S3</t>
   </si>
   <si>
-    <t xml:space="preserve">fu_mic All_literature, high cell permeability, PK-Sim partitioning</t>
+    <t xml:space="preserve">fu_mic all_literature, high cell permeability, PK-Sim partitioning</t>
   </si>
   <si>
     <t xml:space="preserve">high</t>
@@ -325,10 +322,7 @@
     <t xml:space="preserve">S4</t>
   </si>
   <si>
-    <t xml:space="preserve">fu_mic All_literature, high cell permeability, Wood 2017 scaling factors, PK-Sim partitioning</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yes</t>
+    <t xml:space="preserve">fu_mic all_literature, high cell permeability, Wood 2017 scaling factors, PK-Sim partitioning</t>
   </si>
   <si>
     <t xml:space="preserve">S5</t>
@@ -337,7 +331,7 @@
     <t xml:space="preserve">fu_mic Rodgers &amp; Rowland, high cell permeability, Rodgers &amp; Rowland partitioning</t>
   </si>
   <si>
-    <t xml:space="preserve">Rodgers &amp; Rowland + fu</t>
+    <t xml:space="preserve">rodgers_rowland_fu</t>
   </si>
   <si>
     <t xml:space="preserve">single-iv-rodgers-rowland.pkml</t>
@@ -370,7 +364,7 @@
     <t xml:space="preserve"/>
   </si>
   <si>
-    <t xml:space="preserve">Ionization class used by esqIVIVE (acid, base, neutral)</t>
+    <t xml:space="preserve">Ionization class used by ESQivive (acid, base, neutral)</t>
   </si>
   <si>
     <t xml:space="preserve">Most relevant pKa (0 for neutrals)</t>
@@ -457,7 +451,7 @@
     <t xml:space="preserve">Scenario description</t>
   </si>
   <si>
-    <t xml:space="preserve">fu_mic used in IVIVE: none (=1), measured, or any calculate_fu_in_vitro() partition_qspr</t>
+    <t xml:space="preserve">fu_mic used in IVIVE: none (=1), measured, or any calculate_fu_in_vitro() method</t>
   </si>
   <si>
     <t xml:space="preserve">Method used when fu_mic_method fails for a compound (e.g. R&amp;R for non strong bases)</t>
@@ -472,7 +466,7 @@
     <t xml:space="preserve">cm/min</t>
   </si>
   <si>
-    <t xml:space="preserve">Apply Wood 2017 empirical scaling factors in IVIVE_clearance() (Yes / No)</t>
+    <t xml:space="preserve">Apply Wood 2017 empirical scaling factors in ivive_clearance() (TRUE / FALSE)</t>
   </si>
   <si>
     <t xml:space="preserve">Blood/plasma ratio: observed (set blood cell partitioning from BP) or model (PK-Sim formula from LogP)</t>
@@ -2745,13 +2739,13 @@
   <cols>
     <col min="1" max="1" width="8.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="93.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="26.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="18.71" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="15.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="12.71" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="23.71" hidden="0" customWidth="1"/>
-    <col min="7" max="7" width="16.71" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="20.71" hidden="0" customWidth="1"/>
     <col min="8" max="8" width="18.71" hidden="0" customWidth="1"/>
-    <col min="9" max="9" width="22.71" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="30.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2798,149 +2792,149 @@
         <v>92</v>
       </c>
       <c r="F2"/>
-      <c r="G2" t="s">
+      <c r="G2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H2" t="s">
         <v>93</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>94</v>
-      </c>
-      <c r="I2" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
+        <v>95</v>
+      </c>
+      <c r="B3" t="s">
         <v>96</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>97</v>
-      </c>
-      <c r="C3" t="s">
-        <v>98</v>
       </c>
       <c r="D3"/>
       <c r="E3" t="s">
         <v>92</v>
       </c>
       <c r="F3"/>
-      <c r="G3" t="s">
+      <c r="G3" t="b">
+        <v>0</v>
+      </c>
+      <c r="H3" t="s">
         <v>93</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>94</v>
-      </c>
-      <c r="I3" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
+        <v>98</v>
+      </c>
+      <c r="B4" t="s">
         <v>99</v>
       </c>
-      <c r="B4" t="s">
-        <v>100</v>
-      </c>
       <c r="C4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D4"/>
       <c r="E4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F4" t="n">
         <v>1000</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" t="b">
+        <v>0</v>
+      </c>
+      <c r="H4" t="s">
         <v>93</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>94</v>
-      </c>
-      <c r="I4" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
+        <v>101</v>
+      </c>
+      <c r="B5" t="s">
         <v>102</v>
       </c>
-      <c r="B5" t="s">
-        <v>103</v>
-      </c>
       <c r="C5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D5"/>
       <c r="E5" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F5" t="n">
         <v>1000</v>
       </c>
-      <c r="G5" t="s">
-        <v>104</v>
+      <c r="G5" t="b">
+        <v>1</v>
       </c>
       <c r="H5" t="s">
+        <v>93</v>
+      </c>
+      <c r="I5" t="s">
         <v>94</v>
-      </c>
-      <c r="I5" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
+        <v>103</v>
+      </c>
+      <c r="B6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C6" t="s">
         <v>105</v>
       </c>
-      <c r="B6" t="s">
-        <v>106</v>
-      </c>
-      <c r="C6" t="s">
-        <v>107</v>
-      </c>
       <c r="D6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F6" t="n">
         <v>1000</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" t="b">
+        <v>0</v>
+      </c>
+      <c r="H6" t="s">
         <v>93</v>
       </c>
-      <c r="H6" t="s">
-        <v>94</v>
-      </c>
       <c r="I6" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
+        <v>107</v>
+      </c>
+      <c r="B7" t="s">
+        <v>108</v>
+      </c>
+      <c r="C7" t="s">
         <v>109</v>
-      </c>
-      <c r="B7" t="s">
-        <v>110</v>
-      </c>
-      <c r="C7" t="s">
-        <v>111</v>
       </c>
       <c r="D7"/>
       <c r="E7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F7" t="n">
         <v>1000</v>
       </c>
-      <c r="G7" t="s">
+      <c r="G7" t="b">
+        <v>0</v>
+      </c>
+      <c r="H7" t="s">
         <v>93</v>
       </c>
-      <c r="H7" t="s">
+      <c r="I7" t="s">
         <v>94</v>
-      </c>
-      <c r="I7" t="s">
-        <v>95</v>
       </c>
     </row>
   </sheetData>
@@ -2962,436 +2956,436 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>81</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>114</v>
+      </c>
+      <c r="D2" t="s">
         <v>115</v>
-      </c>
-      <c r="B2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" t="s">
-        <v>116</v>
-      </c>
-      <c r="D2" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B3" t="s">
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D3" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B4" t="s">
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D4" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B5" t="s">
         <v>3</v>
       </c>
       <c r="C5" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="D5" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B6" t="s">
         <v>4</v>
       </c>
       <c r="C6" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="D6" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B7" t="s">
         <v>5</v>
       </c>
       <c r="C7" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="D7" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B8" t="s">
         <v>6</v>
       </c>
       <c r="C8" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="D8" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B9" t="s">
         <v>7</v>
       </c>
       <c r="C9" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="D9" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B10" t="s">
         <v>8</v>
       </c>
       <c r="C10" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D10" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B11" t="s">
         <v>9</v>
       </c>
       <c r="C11" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="D11" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B12" t="s">
         <v>10</v>
       </c>
       <c r="C12" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="D12" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B13" t="s">
         <v>11</v>
       </c>
       <c r="C13" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D13" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B14" t="s">
         <v>12</v>
       </c>
       <c r="C14" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="D14" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B15" t="s">
         <v>13</v>
       </c>
       <c r="C15" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D15" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B16" t="s">
         <v>14</v>
       </c>
       <c r="C16" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="D16" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B17" t="s">
         <v>15</v>
       </c>
       <c r="C17" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="D17" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B18" t="s">
         <v>16</v>
       </c>
       <c r="C18" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D18" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B19" t="s">
         <v>17</v>
       </c>
       <c r="C19" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D19" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B20" t="s">
         <v>18</v>
       </c>
       <c r="C20" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D20" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B21" t="s">
         <v>19</v>
       </c>
       <c r="C21" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D21" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B22" t="s">
         <v>20</v>
       </c>
       <c r="C22" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D22" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B23" t="s">
         <v>80</v>
       </c>
       <c r="C23" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D23" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B24" t="s">
         <v>81</v>
       </c>
       <c r="C24" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D24" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B25" t="s">
         <v>82</v>
       </c>
       <c r="C25" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D25" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B26" t="s">
         <v>83</v>
       </c>
       <c r="C26" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="D26" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B27" t="s">
         <v>84</v>
       </c>
       <c r="C27" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="D27" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B28" t="s">
         <v>85</v>
       </c>
       <c r="C28" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D28" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B29" t="s">
         <v>86</v>
       </c>
       <c r="C29" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D29" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B30" t="s">
         <v>87</v>
       </c>
       <c r="C30" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="D30" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B31" t="s">
         <v>88</v>
       </c>
       <c r="C31" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="D31" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
   </sheetData>

</xml_diff>